<commit_message>
Correct enhancement prices to configured exponential growth
Keep first purchase100: target L costs cost_base * cost_growth^(L-1), default growth3. Use bounded GrowthNumber geometric totals and existing MAX binary search; retain saves, purchased levels, balances and branches.
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/enhance_config.xlsx
+++ b/space-battleship/config_excel/enhance_config.xlsx
@@ -331,21 +331,21 @@
         <x:v>碎片</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>费用系数；正整数碎片数</x:v>
+        <x:v>首级费用；正整数碎片数</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" t="str">
-        <x:v>cost_exponent</x:v>
+        <x:v>cost_growth</x:v>
       </x:c>
       <x:c r="B5" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>次方</x:v>
+        <x:v>倍率</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>整数0..16；费用＝系数×目标实际等级^指数</x:v>
+        <x:v>整数≥1；费用＝首级费用×倍率^(购买等级−1)</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">

</xml_diff>

<commit_message>
Gate shared enhancement effects and branches by rank and expose exact details
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/enhance_config.xlsx
+++ b/space-battleship/config_excel/enhance_config.xlsx
@@ -463,16 +463,16 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>装备级</t>
+          <t>强化级</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第一顺位生效的实际装备等级</t>
+          <t>第1顺位效果的有效共享强化等级门槛；装备等级无关</t>
         </is>
       </c>
     </row>
@@ -483,16 +483,16 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>装备级</t>
+          <t>强化级</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第二顺位生效的实际装备等级</t>
+          <t>第2顺位效果的有效共享强化等级门槛；装备等级无关</t>
         </is>
       </c>
     </row>
@@ -503,16 +503,16 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>装备级</t>
+          <t>强化级</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第三顺位生效的实际装备等级</t>
+          <t>第3顺位效果的有效共享强化等级门槛；装备等级无关</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>每种效果第一分支节点的解锁等级</t>
+          <t>第1分支节点基础门槛；加上效果当前位置的有效共享强化门槛</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>每种效果第二分支节点的解锁等级</t>
+          <t>第2分支节点基础门槛；加上效果当前位置的有效共享强化门槛</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>每种效果第三分支节点的解锁等级</t>
+          <t>第3分支节点基础门槛；加上效果当前位置的有效共享强化门槛</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gate enhancement consumers and separate effect and branch thresholds
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/enhance_config.xlsx
+++ b/space-battleship/config_excel/enhance_config.xlsx
@@ -341,7 +341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -892,7 +892,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第1分支节点基础门槛；加上效果当前位置的有效共享强化门槛</t>
+          <t>分支节点基础门槛；加上独立的效果位置偏移，不加主效果启用门槛</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第2分支节点基础门槛；加上效果当前位置的有效共享强化门槛</t>
+          <t>分支节点基础门槛；加上独立的效果位置偏移，不加主效果启用门槛</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第3分支节点基础门槛；加上效果当前位置的有效共享强化门槛</t>
+          <t>分支节点基础门槛；加上独立的效果位置偏移，不加主效果启用门槛</t>
         </is>
       </c>
     </row>
@@ -1713,6 +1713,66 @@
       <c r="D68" t="inlineStr">
         <is>
           <t>未强制清除概率缺口转化为伤害增加的系数</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>branch_position_offset_1</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>有效强化级</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>第1顺位分支门槛偏移；与主效果启用门槛独立</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>branch_position_offset_2</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>10</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>有效强化级</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>第2顺位分支门槛偏移；与主效果启用门槛独立</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>branch_position_offset_3</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>20</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>有效强化级</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>第3顺位分支门槛偏移；与主效果启用门槛独立</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: slow memory repair and limit stored protection
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/enhance_config.xlsx
+++ b/space-battleship/config_excel/enhance_config.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="enhance_config" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="enhance_config" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>0.01</v>
+        <v>0.0005</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: defer global memory rate changes from opening scope
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/enhance_config.xlsx
+++ b/space-battleship/config_excel/enhance_config.xlsx
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>0.0005</v>
+        <v>0.01</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rebuild stage 1 configuration, Amount, native headless and save foundation
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/enhance_config.xlsx
+++ b/space-battleship/config_excel/enhance_config.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>所有我方武器基础暴击率；0.25＝25%</t>
+          <t>The active critical enhancement supplies 25%; weapons have no innate critical chance.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>普通连发后允许额外再触发的连发次数</t>
+          <t>Additional attacks do not trigger repeat fire.</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>保底暴击的实际暴击概率；默认必定</t>
+          <t>Guarantee critical effects; extra critical damage still uses the original chance, excluding drone chance.</t>
         </is>
       </c>
     </row>

</xml_diff>